<commit_message>
add descriptions and more results
</commit_message>
<xml_diff>
--- a/results/Literature validation.xlsx
+++ b/results/Literature validation.xlsx
@@ -1,44 +1,44 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cheți\Documents\Doctorate\Doctorate 2022\Daiana\Drug-Disease networks\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cheți\Documents\Doctorate\Doctorate 2022\Daiana\Drug-Disease networks\Frontiers Bioinfo\Revision 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84AF1FE0-66AE-43AD-9907-904923A8175F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D1CA001-6C59-4071-869C-6EB4960F60AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="836" firstSheet="3" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="836" firstSheet="4" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Comm 1_N" sheetId="1" r:id="rId1"/>
-    <sheet name="Comm2_B" sheetId="2" r:id="rId2"/>
-    <sheet name="Comm3_C" sheetId="3" r:id="rId3"/>
-    <sheet name="Comm4_L" sheetId="4" r:id="rId4"/>
-    <sheet name="Comm5_D" sheetId="5" r:id="rId5"/>
-    <sheet name="Comm6_L" sheetId="6" r:id="rId6"/>
-    <sheet name="Comm7_M" sheetId="7" r:id="rId7"/>
-    <sheet name="Comm8_G" sheetId="8" r:id="rId8"/>
-    <sheet name="Comm9_N" sheetId="9" r:id="rId9"/>
-    <sheet name="Comm10_L" sheetId="10" r:id="rId10"/>
-    <sheet name="Comm11_H" sheetId="11" r:id="rId11"/>
-    <sheet name="Comm12_D" sheetId="12" r:id="rId12"/>
+    <sheet name="community 1_N" sheetId="1" r:id="rId1"/>
+    <sheet name="community 2_B" sheetId="2" r:id="rId2"/>
+    <sheet name="community 3_C" sheetId="3" r:id="rId3"/>
+    <sheet name="community 4_L" sheetId="4" r:id="rId4"/>
+    <sheet name="community 5_D" sheetId="5" r:id="rId5"/>
+    <sheet name="community 6_L" sheetId="6" r:id="rId6"/>
+    <sheet name="community 7_M" sheetId="7" r:id="rId7"/>
+    <sheet name="community 8_G" sheetId="8" r:id="rId8"/>
+    <sheet name="community 9_N" sheetId="9" r:id="rId9"/>
+    <sheet name="community 10_L" sheetId="10" r:id="rId10"/>
+    <sheet name="community 11_H" sheetId="11" r:id="rId11"/>
+    <sheet name="community 12_D" sheetId="12" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Comm 1_N'!$A$1:$E$65</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">Comm10_L!$A$1:$E$1003</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">Comm11_H!$A$1:$E$1003</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">Comm12_D!$A$1:$E$1002</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Comm2_B!$A$1:$E$46</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Comm3_C!$A$1:$E$68</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Comm4_L!$A$1:$E$64</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Comm5_D!$A$1:$E$1008</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Comm6_L!$A$1:$E$1008</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Comm7_M!$A$1:$E$1001</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Comm8_G!$A$1:$E$1003</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Comm9_N!$A$1:$E$1004</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'community 1_N'!$A$1:$E$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'community 10_L'!$A$1:$E$1003</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'community 11_H'!$A$1:$E$1003</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'community 12_D'!$A$1:$E$1002</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'community 2_B'!$A$1:$E$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'community 3_C'!$A$1:$E$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'community 4_L'!$A$1:$E$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'community 5_D'!$A$1:$E$1008</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'community 6_L'!$A$1:$E$1008</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'community 7_M'!$A$1:$E$1001</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'community 8_G'!$A$1:$E$1003</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'community 9_N'!$A$1:$E$1004</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -60,165 +60,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author/>
-  </authors>
-  <commentList>
-    <comment ref="C45" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>======
-ID#AAABQE7fpBU
-Daiana Hânda    (2024-06-19 15:19:27)
-cod nou ATC v. 2024</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-  <extLst>
-    <ext xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mj10NhyGUfZwKpWck7QbXtQcCpbsg=="/>
-    </ext>
-  </extLst>
-</comments>
-</file>
-
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author/>
-  </authors>
-  <commentList>
-    <comment ref="C46" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>======
-ID#AAABQE7fpBY
-Daiana Hânda    (2024-06-19 15:36:32)
-cod nou ATC v. 2024</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-  <extLst>
-    <ext xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mgDXBMl7ztEkkPFwm5WVy3Qv+0WFQ=="/>
-    </ext>
-  </extLst>
-</comments>
-</file>
-
-<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author/>
-  </authors>
-  <commentList>
-    <comment ref="C9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000003000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>======
-ID#AAABQE7fpBc
-Daiana Hânda    (2024-06-19 15:40:44)
-diferenta fata de retea</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C26" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>======
-ID#AAABQE7fpBo
-Daiana Hânda    (2024-06-19 15:44:40)
-diferenta fata de retea</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C49" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>======
-ID#AAABQE7fpBs
-Daiana Hânda    (2024-06-19 15:50:58)
-diferenta fata de retea</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-  <extLst>
-    <ext xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mj6lmxUm4K/cN2n8OaN9TzraazUMA=="/>
-    </ext>
-  </extLst>
-</comments>
-</file>
-
-<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author/>
-  </authors>
-  <commentList>
-    <comment ref="B56" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>======
-ID#AAABMcI4-qA
-Lucretia Udrescu    (2024-04-24 10:33:39)
-https://www.nature.com/articles/cdd200812
-"In genetic models, HIF-1α has been identified as a positive factor for tumor growth43 and increased HIF-1α activation was also correlated with the development of a more aggressive phenotype in a model of epidermal carcinogenesis.49"</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-  <extLst>
-    <ext xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7miTBuBYaLqsxCoicGhoJzl0hPNE1Q=="/>
-    </ext>
-  </extLst>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="872" uniqueCount="575">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="871" uniqueCount="575">
   <si>
     <t>Drugname</t>
   </si>
@@ -2094,39 +1937,35 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -2343,7 +2182,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E1014"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
@@ -3243,11 +3082,11 @@
         <v>2017</v>
       </c>
     </row>
-    <row r="66" spans="1:5" s="27" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="67" spans="1:5" s="27" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="68" spans="1:5" s="27" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="69" spans="1:5" s="27" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="70" spans="1:5" s="27" customFormat="1" ht="15.75" customHeight="1"/>
+    <row r="66" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="67" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="68" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="69" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="70" spans="1:5" ht="15.75" customHeight="1"/>
     <row r="71" spans="1:5" ht="15.75" customHeight="1"/>
     <row r="72" spans="1:5" ht="15.75" customHeight="1"/>
     <row r="73" spans="1:5" ht="15.75" customHeight="1"/>
@@ -4239,8 +4078,7 @@
     <hyperlink ref="D65" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
-  <legacyDrawing r:id="rId43"/>
+  <pageSetup orientation="landscape" r:id="rId43"/>
 </worksheet>
 </file>
 
@@ -4344,21 +4182,15 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="9" spans="1:5" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="10" spans="1:5" s="24" customFormat="1" ht="14.4">
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-    </row>
-    <row r="11" spans="1:5" s="24" customFormat="1" ht="14.4">
-      <c r="B11" s="28"/>
-      <c r="C11" s="28"/>
-    </row>
-    <row r="12" spans="1:5" s="24" customFormat="1" ht="14.4"/>
-    <row r="13" spans="1:5" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="14" spans="1:5" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="15" spans="1:5" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="16" spans="1:5" s="24" customFormat="1" ht="15" customHeight="1"/>
+    <row r="10" spans="1:5" ht="14.4">
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+    </row>
+    <row r="11" spans="1:5" ht="14.4">
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
+    </row>
+    <row r="12" spans="1:5" ht="14.4"/>
     <row r="24" ht="15.75" customHeight="1"/>
     <row r="25" ht="15.75" customHeight="1"/>
     <row r="26" ht="15.75" customHeight="1"/>
@@ -5348,7 +5180,7 @@
     <hyperlink ref="D5" r:id="rId4" xr:uid="{00000000-0004-0000-0900-000008000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
+  <pageSetup orientation="landscape" r:id="rId5"/>
 </worksheet>
 </file>
 
@@ -5411,11 +5243,9 @@
       <c r="B4" s="11" t="s">
         <v>545</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
     </row>
     <row r="5" spans="1:6" ht="19.2">
       <c r="A5" s="12">
@@ -5424,16 +5254,16 @@
       <c r="B5" s="10" t="s">
         <v>546</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="16" t="s">
         <v>547</v>
       </c>
-      <c r="E5" s="24">
+      <c r="E5" s="12">
         <v>2011</v>
       </c>
-      <c r="F5" s="26"/>
+      <c r="F5" s="23"/>
     </row>
     <row r="6" spans="1:6" ht="14.4">
       <c r="A6" s="12">
@@ -5442,13 +5272,13 @@
       <c r="B6" s="10" t="s">
         <v>548</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="25" t="s">
+      <c r="D6" s="16" t="s">
         <v>549</v>
       </c>
-      <c r="E6" s="24">
+      <c r="E6" s="12">
         <v>2020</v>
       </c>
     </row>
@@ -5508,21 +5338,15 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:6" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="15" spans="1:6" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="16" spans="1:6" s="24" customFormat="1" ht="14.4">
-      <c r="B16" s="22"/>
-      <c r="C16" s="22"/>
-    </row>
-    <row r="17" spans="2:3" s="24" customFormat="1" ht="14.4">
-      <c r="B17" s="28"/>
-      <c r="C17" s="28"/>
-    </row>
-    <row r="18" spans="2:3" s="24" customFormat="1" ht="14.4"/>
-    <row r="19" spans="2:3" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="20" spans="2:3" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="21" spans="2:3" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="22" spans="2:3" s="24" customFormat="1" ht="15" customHeight="1"/>
+    <row r="16" spans="1:6" ht="14.4">
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+    </row>
+    <row r="17" spans="2:3" ht="14.4">
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
+    </row>
+    <row r="18" spans="2:3" ht="14.4"/>
     <row r="24" spans="2:3" ht="15.75" customHeight="1"/>
     <row r="25" spans="2:3" ht="15.75" customHeight="1"/>
     <row r="26" spans="2:3" ht="15.75" customHeight="1"/>
@@ -6510,7 +6334,7 @@
     <hyperlink ref="D6" r:id="rId2" xr:uid="{00000000-0004-0000-0A00-000003000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
+  <pageSetup orientation="landscape" r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -6699,19 +6523,15 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="13" spans="1:5" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="14" spans="1:5" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="15" spans="1:5" s="24" customFormat="1" ht="14.4">
-      <c r="B15" s="22"/>
-      <c r="C15" s="22"/>
-    </row>
-    <row r="16" spans="1:5" s="24" customFormat="1" ht="14.4">
-      <c r="B16" s="28"/>
-      <c r="C16" s="28"/>
-    </row>
-    <row r="17" s="24" customFormat="1" ht="14.4"/>
-    <row r="18" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="19" s="24" customFormat="1" ht="15" customHeight="1"/>
+    <row r="15" spans="1:5" ht="14.4">
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+    </row>
+    <row r="16" spans="1:5" ht="14.4">
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+    </row>
+    <row r="17" ht="14.4"/>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="15.75" customHeight="1"/>
     <row r="25" ht="15.75" customHeight="1"/>
@@ -7705,16 +7525,16 @@
     <hyperlink ref="D12" r:id="rId8" xr:uid="{00000000-0004-0000-0B00-00000F000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
+  <pageSetup orientation="landscape" r:id="rId9"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5.33203125" style="12" customWidth="1"/>
@@ -8312,12 +8132,9 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="48" spans="1:5" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="49" s="24" customFormat="1" ht="14.4"/>
-    <row r="50" s="24" customFormat="1" ht="14.4"/>
-    <row r="51" s="24" customFormat="1" ht="14.4"/>
-    <row r="52" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="53" s="24" customFormat="1" ht="15" customHeight="1"/>
+    <row r="49" ht="14.4"/>
+    <row r="50" ht="14.4"/>
+    <row r="51" ht="14.4"/>
   </sheetData>
   <autoFilter ref="A1:E46" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <hyperlinks>
@@ -8339,13 +8156,12 @@
     <hyperlink ref="D46" r:id="rId16" xr:uid="{00000000-0004-0000-0100-00001E000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
-  <legacyDrawing r:id="rId17"/>
+  <pageSetup orientation="landscape" r:id="rId17"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E1005"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
@@ -9187,13 +9003,13 @@
         <v>4</v>
       </c>
     </row>
-    <row r="69" spans="1:3" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="70" spans="1:3" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="71" spans="1:3" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="72" spans="1:3" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="73" spans="1:3" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="74" spans="1:3" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="75" spans="1:3" s="24" customFormat="1" ht="15.75" customHeight="1"/>
+    <row r="69" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="70" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="71" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="72" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="73" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="74" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="75" spans="1:3" ht="15.75" customHeight="1"/>
     <row r="76" spans="1:3" ht="15.75" customHeight="1"/>
     <row r="77" spans="1:3" ht="15.75" customHeight="1"/>
     <row r="78" spans="1:3" ht="15.75" customHeight="1"/>
@@ -10148,20 +9964,19 @@
     <hyperlink ref="D53" r:id="rId19" xr:uid="{00000000-0004-0000-0200-000025000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
-  <legacyDrawing r:id="rId20"/>
+  <pageSetup orientation="landscape" r:id="rId20"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E1023"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:E1022"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="6" style="12" customWidth="1"/>
     <col min="2" max="2" width="18.33203125" style="12" customWidth="1"/>
     <col min="3" max="3" width="17" style="12" customWidth="1"/>
-    <col min="4" max="4" width="17.77734375" style="12" customWidth="1"/>
+    <col min="4" max="4" width="30.109375" style="12" customWidth="1"/>
     <col min="5" max="5" width="7.88671875" style="12" customWidth="1"/>
     <col min="6" max="21" width="10.6640625" style="12" customWidth="1"/>
     <col min="22" max="16384" width="14.44140625" style="12"/>
@@ -10901,8 +10716,15 @@
       </c>
     </row>
     <row r="57" spans="1:5" ht="15.75" customHeight="1">
-      <c r="B57" s="11"/>
-      <c r="C57" s="11"/>
+      <c r="A57" s="12">
+        <v>35</v>
+      </c>
+      <c r="B57" s="10" t="s">
+        <v>350</v>
+      </c>
+      <c r="C57" s="11" t="s">
+        <v>26</v>
+      </c>
       <c r="D57" s="16" t="s">
         <v>349</v>
       </c>
@@ -10912,10 +10734,10 @@
     </row>
     <row r="58" spans="1:5" ht="15.75" customHeight="1">
       <c r="A58" s="12">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C58" s="11" t="s">
         <v>26</v>
@@ -10929,41 +10751,41 @@
     </row>
     <row r="59" spans="1:5" ht="15.75" customHeight="1">
       <c r="A59" s="12">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C59" s="11" t="s">
         <v>26</v>
       </c>
       <c r="D59" s="16" t="s">
+        <v>353</v>
+      </c>
+      <c r="E59" s="12">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="15.75" customHeight="1">
+      <c r="B60" s="11"/>
+      <c r="C60" s="11"/>
+      <c r="D60" s="16" t="s">
         <v>349</v>
       </c>
-      <c r="E59" s="12">
+      <c r="E60" s="12">
         <v>2005</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A60" s="12">
-        <v>37</v>
-      </c>
-      <c r="B60" s="10" t="s">
-        <v>352</v>
-      </c>
-      <c r="C60" s="11" t="s">
+    <row r="61" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A61" s="12">
+        <v>38</v>
+      </c>
+      <c r="B61" s="10" t="s">
+        <v>354</v>
+      </c>
+      <c r="C61" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="D60" s="16" t="s">
-        <v>353</v>
-      </c>
-      <c r="E60" s="12">
-        <v>2015</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" ht="15.75" customHeight="1">
-      <c r="B61" s="11"/>
-      <c r="C61" s="11"/>
       <c r="D61" s="16" t="s">
         <v>349</v>
       </c>
@@ -10973,50 +10795,34 @@
     </row>
     <row r="62" spans="1:5" ht="15.75" customHeight="1">
       <c r="A62" s="12">
-        <v>38</v>
-      </c>
-      <c r="B62" s="10" t="s">
-        <v>354</v>
+        <v>39</v>
+      </c>
+      <c r="B62" s="11" t="s">
+        <v>355</v>
       </c>
       <c r="C62" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="D62" s="16" t="s">
-        <v>349</v>
-      </c>
-      <c r="E62" s="12">
-        <v>2005</v>
-      </c>
     </row>
     <row r="63" spans="1:5" ht="15.75" customHeight="1">
       <c r="A63" s="12">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B63" s="11" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C63" s="11" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A64" s="12">
-        <v>40</v>
-      </c>
-      <c r="B64" s="11" t="s">
-        <v>356</v>
-      </c>
-      <c r="C64" s="11" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="65" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="66" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="67" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="68" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="69" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="70" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="71" s="24" customFormat="1" ht="15.75" customHeight="1"/>
+    <row r="64" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="65" ht="15.75" customHeight="1"/>
+    <row r="66" ht="15.75" customHeight="1"/>
+    <row r="67" ht="15.75" customHeight="1"/>
+    <row r="68" ht="15.75" customHeight="1"/>
+    <row r="69" ht="15.75" customHeight="1"/>
+    <row r="70" ht="15.75" customHeight="1"/>
+    <row r="71" ht="15.75" customHeight="1"/>
     <row r="72" ht="15.75" customHeight="1"/>
     <row r="73" ht="15.75" customHeight="1"/>
     <row r="74" ht="15.75" customHeight="1"/>
@@ -11968,9 +11774,8 @@
     <row r="1020" ht="15.75" customHeight="1"/>
     <row r="1021" ht="15.75" customHeight="1"/>
     <row r="1022" ht="15.75" customHeight="1"/>
-    <row r="1023" ht="15.75" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A1:E64" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <autoFilter ref="A1:E63" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <hyperlinks>
     <hyperlink ref="D3" r:id="rId1" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
     <hyperlink ref="D5" r:id="rId2" xr:uid="{00000000-0004-0000-0300-000003000000}"/>
@@ -12015,16 +11820,14 @@
     <hyperlink ref="D50" r:id="rId41" xr:uid="{00000000-0004-0000-0300-000051000000}"/>
     <hyperlink ref="D55" r:id="rId42" xr:uid="{00000000-0004-0000-0300-000053000000}"/>
     <hyperlink ref="D56" r:id="rId43" xr:uid="{00000000-0004-0000-0300-000055000000}"/>
-    <hyperlink ref="D57" r:id="rId44" xr:uid="{00000000-0004-0000-0300-000057000000}"/>
-    <hyperlink ref="D58" r:id="rId45" xr:uid="{00000000-0004-0000-0300-000059000000}"/>
-    <hyperlink ref="D59" r:id="rId46" xr:uid="{00000000-0004-0000-0300-00005B000000}"/>
-    <hyperlink ref="D60" r:id="rId47" xr:uid="{00000000-0004-0000-0300-00005D000000}"/>
-    <hyperlink ref="D61" r:id="rId48" xr:uid="{00000000-0004-0000-0300-00005F000000}"/>
-    <hyperlink ref="D62" r:id="rId49" xr:uid="{00000000-0004-0000-0300-000061000000}"/>
+    <hyperlink ref="D57" r:id="rId44" xr:uid="{00000000-0004-0000-0300-000059000000}"/>
+    <hyperlink ref="D58" r:id="rId45" xr:uid="{00000000-0004-0000-0300-00005B000000}"/>
+    <hyperlink ref="D59" r:id="rId46" xr:uid="{00000000-0004-0000-0300-00005D000000}"/>
+    <hyperlink ref="D60" r:id="rId47" xr:uid="{00000000-0004-0000-0300-00005F000000}"/>
+    <hyperlink ref="D61" r:id="rId48" xr:uid="{00000000-0004-0000-0300-000061000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
-  <legacyDrawing r:id="rId50"/>
+  <pageSetup orientation="landscape" r:id="rId49"/>
 </worksheet>
 </file>
 
@@ -12426,19 +12229,19 @@
         <v>34</v>
       </c>
     </row>
-    <row r="31" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1">
-      <c r="B31" s="22"/>
-      <c r="C31" s="22"/>
-    </row>
-    <row r="32" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1">
-      <c r="B32" s="22"/>
-      <c r="C32" s="22"/>
-    </row>
-    <row r="33" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="34" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="35" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="36" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="37" s="24" customFormat="1" ht="15.75" customHeight="1"/>
+    <row r="31" spans="1:5" ht="15.75" customHeight="1">
+      <c r="B31" s="11"/>
+      <c r="C31" s="11"/>
+    </row>
+    <row r="32" spans="1:5" ht="15.75" customHeight="1">
+      <c r="B32" s="11"/>
+      <c r="C32" s="11"/>
+    </row>
+    <row r="33" ht="15.75" customHeight="1"/>
+    <row r="34" ht="15.75" customHeight="1"/>
+    <row r="35" ht="15.75" customHeight="1"/>
+    <row r="36" ht="15.75" customHeight="1"/>
+    <row r="37" ht="15.75" customHeight="1"/>
     <row r="38" ht="15.75" customHeight="1"/>
     <row r="39" ht="15.75" customHeight="1"/>
     <row r="40" ht="15.75" customHeight="1"/>
@@ -13430,7 +13233,7 @@
     <hyperlink ref="D29" r:id="rId15" xr:uid="{00000000-0004-0000-0400-00001E000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
+  <pageSetup orientation="landscape" r:id="rId16"/>
 </worksheet>
 </file>
 
@@ -13838,13 +13641,13 @@
         <v>170</v>
       </c>
     </row>
-    <row r="30" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="31" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="32" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="33" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="34" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="35" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="36" s="24" customFormat="1" ht="15.75" customHeight="1"/>
+    <row r="30" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="31" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="32" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="33" ht="15.75" customHeight="1"/>
+    <row r="34" ht="15.75" customHeight="1"/>
+    <row r="35" ht="15.75" customHeight="1"/>
+    <row r="36" ht="15.75" customHeight="1"/>
     <row r="37" ht="15.6" customHeight="1"/>
     <row r="38" ht="15.75" customHeight="1"/>
     <row r="39" ht="15.75" customHeight="1"/>
@@ -14842,7 +14645,7 @@
     <hyperlink ref="D26" r:id="rId20" xr:uid="{00000000-0004-0000-0500-000027000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
+  <pageSetup orientation="landscape" r:id="rId21"/>
 </worksheet>
 </file>
 
@@ -15134,18 +14937,17 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:5" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="22" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="23" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="24" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="25" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="26" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="27" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="28" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="29" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="30" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="31" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="32" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1"/>
+    <row r="22" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="23" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="24" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="25" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="26" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="27" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="28" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="29" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="30" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="31" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="32" spans="1:5" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>
@@ -16129,7 +15931,7 @@
     <hyperlink ref="D17" r:id="rId9" xr:uid="{00000000-0004-0000-0600-000011000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
+  <pageSetup orientation="landscape" r:id="rId10"/>
 </worksheet>
 </file>
 
@@ -16371,7 +16173,7 @@
       <c r="C16" s="11" t="s">
         <v>503</v>
       </c>
-      <c r="D16" s="22"/>
+      <c r="D16" s="11"/>
     </row>
     <row r="17" spans="1:5" ht="14.4">
       <c r="A17" s="12">
@@ -16433,26 +16235,24 @@
         <v>77</v>
       </c>
     </row>
-    <row r="22" spans="1:5" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="23" spans="1:5" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="24" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1">
-      <c r="B24" s="22"/>
-      <c r="C24" s="22"/>
-    </row>
-    <row r="25" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1">
-      <c r="B25" s="28"/>
-      <c r="C25" s="28"/>
-    </row>
-    <row r="26" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="27" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="28" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1">
-      <c r="B28" s="29"/>
-    </row>
-    <row r="29" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1">
-      <c r="B29" s="29"/>
-    </row>
-    <row r="30" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1"/>
-    <row r="31" spans="1:5" s="24" customFormat="1" ht="15.75" customHeight="1"/>
+    <row r="24" spans="1:5" ht="15.75" customHeight="1">
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+    </row>
+    <row r="25" spans="1:5" ht="15.75" customHeight="1">
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
+    </row>
+    <row r="26" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="27" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="28" spans="1:5" ht="15.75" customHeight="1">
+      <c r="B28" s="25"/>
+    </row>
+    <row r="29" spans="1:5" ht="15.75" customHeight="1">
+      <c r="B29" s="25"/>
+    </row>
+    <row r="30" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="31" spans="1:5" ht="15.75" customHeight="1"/>
     <row r="32" spans="1:5" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="15.75" customHeight="1"/>
@@ -17441,7 +17241,7 @@
     <hyperlink ref="D18" r:id="rId11" xr:uid="{00000000-0004-0000-0700-000011000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
+  <pageSetup orientation="landscape" r:id="rId12"/>
 </worksheet>
 </file>
 
@@ -17479,7 +17279,7 @@
       <c r="A2" s="12">
         <v>1</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="22" t="s">
         <v>511</v>
       </c>
       <c r="C2" s="11" t="s">
@@ -17677,19 +17477,15 @@
         <v>535</v>
       </c>
     </row>
-    <row r="18" spans="1:3" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="19" spans="1:3" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="20" spans="1:3" s="24" customFormat="1" ht="14.4">
-      <c r="B20" s="22"/>
-      <c r="C20" s="22"/>
-    </row>
-    <row r="21" spans="1:3" s="24" customFormat="1" ht="14.4">
-      <c r="B21" s="28"/>
-      <c r="C21" s="28"/>
-    </row>
-    <row r="22" spans="1:3" s="24" customFormat="1" ht="14.4"/>
-    <row r="23" spans="1:3" s="24" customFormat="1" ht="15" customHeight="1"/>
-    <row r="24" spans="1:3" s="24" customFormat="1" ht="15" customHeight="1"/>
+    <row r="20" spans="1:3" ht="14.4">
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+    </row>
+    <row r="21" spans="1:3" ht="14.4">
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
+    </row>
+    <row r="22" spans="1:3" ht="14.4"/>
     <row r="25" spans="1:3" ht="15.75" customHeight="1"/>
     <row r="26" spans="1:3" ht="15.75" customHeight="1"/>
     <row r="27" spans="1:3" ht="15.75" customHeight="1"/>
@@ -18684,6 +18480,6 @@
     <hyperlink ref="D16" r:id="rId9" xr:uid="{00000000-0004-0000-0800-000011000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
+  <pageSetup orientation="landscape" r:id="rId10"/>
 </worksheet>
 </file>
</xml_diff>